<commit_message>
fih labots ieņemuma tips
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/bilance_2026-2027.xlsx
+++ b/bilance_2026-2027.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,15 +486,111 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ienemumi kopa EUR</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+          <t>member_fee</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Juris Radus</t>
+        </is>
+      </c>
       <c r="C4" t="n">
-        <v>430</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+        <v>260</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Biedra naudas iemaksa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>member_fee</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lauris Alainis</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>130</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Biedra naudas iemaksa</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>member_fee</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Oskars Čodors</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Biedra naudas iemaksa</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="n">
+        <v>35</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Viesmednieks</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ienemumi kopā EUR</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="n">
+        <v>865</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -507,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -565,15 +661,78 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Izdevumi kopa EUR</t>
+          <t>Saimnieciskie izdevumi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>450</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+        <v>35</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>naglas un citi būvniecības materiāli</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nodokļi</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>232</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>zemes nodoklis</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Bebru uzraudzības izdevumi</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>jaunas lamatas</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Izdevumi kopā EUR</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>720.0599999999999</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -592,7 +751,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Parskata periods</t>
+          <t>Pārskata periods</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -604,11 +763,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ienemumi EUR</t>
+          <t>Ieņēmumi EUR</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>430</v>
+        <v>865</v>
       </c>
     </row>
     <row r="3">
@@ -618,17 +777,17 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>450</v>
+        <v>720.0599999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Deficits EUR</t>
+          <t>Atlikums EUR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-20</v>
+        <v>144.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>